<commit_message>
feat(map): SkydivePyramid 맵 행(id 9)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#Map.xlsx
+++ b/table/Datas/#Map.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -712,6 +712,29 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SkydivePyramid</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>하늘 피라미드</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Assets/Art/Scenes/SkydivePyramidMap.unity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(map): SkydiveChimney 굴뚝 시제품 맵 행(id 10)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#Map.xlsx
+++ b/table/Datas/#Map.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -735,6 +735,29 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SkydiveChimney</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>굴뚝 시제품</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Assets/Art/Scenes/SkydiveChimneyMap.unity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(map): SkydiveSpiral 피라미드 개정안 맵 행(id 11)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#Map.xlsx
+++ b/table/Datas/#Map.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -758,6 +758,29 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="B15" t="n">
+        <v>11</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SkydiveSpiral</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>피라미드 개정안</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Assets/Art/Scenes/SkydiveSpiralMap.unity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(map): SkydiveCylinder 원통 시제품 맵 행(id 12)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J3Xe7rZoLKi3dJFGKrLsGL
</commit_message>
<xml_diff>
--- a/table/Datas/#Map.xlsx
+++ b/table/Datas/#Map.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -781,6 +781,29 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="B16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C16" t="n">
+        <v>8</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SkydiveCylinder</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>원통 시제품</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Assets/Art/Scenes/SkydiveCylinderMap.unity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>